<commit_message>
Refresh the equipment Excel so Control is a Sí/No dropdown.
Same 99 current nodes; Control no longer uses the multi-status list.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -561,7 +561,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -575,7 +575,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 26/08/2026 16:40 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
+          <t>Equipos vigentes al 26/08/2026 16:59 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       <formula1>"Sí,No,Pendiente"</formula1>
     </dataValidation>
     <dataValidation sqref="F5:F103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Control" error="Elija una opción de la lista (o borre la celda)." promptTitle="Control" prompt="Seleccione un valor para Control o déjelo en blanco" type="list">
-      <formula1>"Pendiente,Revisado OK,En cero,Sin datos,Fuera de servicio,Observación"</formula1>
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2937,7 +2937,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 16:40 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 16:59 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>26/08/2026 16:40 hora Chile</t>
+          <t>26/08/2026 16:59 hora Chile</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Columna para completar al revisar: Pendiente, Revisado OK, En cero, Sin datos, Fuera de servicio u Observación.</t>
+          <t>Columna para completar: Sí o No. Use el desplegable o déjela en blanco.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add BUPA Antofagasta to the current equipment Excel.
Four operational nodes (000029-07..10) appear as client BUPA Antofagasta; Control remains Sí/No. Snapshot is 103 vigentes.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Cómo usar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equipos vigentes'!$A$4:$G$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equipos vigentes'!$A$4:$G$107</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Equipos vigentes'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen por cliente'!$A$4:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen por cliente'!$A$4:$C$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 26/08/2026 16:59 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
+          <t>Equipos vigentes al 26/08/2026 17:04 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
         </is>
       </c>
     </row>
@@ -737,17 +737,17 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA Antofagasta</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>000021-05</t>
+          <t>000029-09</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Calle de Servicio</t>
+          <t>Medidor Principal Sanitaria</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
@@ -760,17 +760,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA Antofagasta</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>000021-07</t>
+          <t>000029-10</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Canchas de Tenis</t>
+          <t>Sala de Bomba N°2</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
@@ -783,17 +783,17 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA Antofagasta</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>000021-01</t>
+          <t>000029-07</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Club House CDUC</t>
+          <t>Sala de Bomba Principal</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
@@ -806,17 +806,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA Antofagasta</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>000021-04</t>
+          <t>000029-08</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Equitación</t>
+          <t>Sala de Bomba Sexto Piso</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
@@ -834,12 +834,12 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>000021-03</t>
+          <t>000021-05</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Raimundo Tupper</t>
+          <t>Calle de Servicio</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
@@ -852,17 +852,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>000009-00</t>
+          <t>000021-07</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Copec Costanera</t>
+          <t>Canchas de Tenis</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
@@ -875,17 +875,17 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>000009-09</t>
+          <t>000021-01</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Copec Lavado Auto servicio Norte</t>
+          <t>Club House CDUC</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
@@ -898,17 +898,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>000009-10</t>
+          <t>000021-04</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Copec Lavado Auto servicio Sur</t>
+          <t>Equitación</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
@@ -921,17 +921,17 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>000009-06</t>
+          <t>000021-03</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Copec Matriz Principal</t>
+          <t>Raimundo Tupper</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr"/>
@@ -949,12 +949,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>000009-08</t>
+          <t>000009-00</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Copec Pronto Baños</t>
+          <t>Copec Costanera</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr"/>
@@ -972,12 +972,12 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>000009-11</t>
+          <t>000009-09</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Copec Pronto Tienda</t>
+          <t>Copec Lavado Auto servicio Norte</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr"/>
@@ -995,12 +995,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>000009-05</t>
+          <t>000009-10</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Copec Riego</t>
+          <t>Copec Lavado Auto servicio Sur</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
@@ -1018,12 +1018,12 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>000009-02</t>
+          <t>000009-06</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Estanque Reutilización</t>
+          <t>Copec Matriz Principal</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr"/>
@@ -1041,12 +1041,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>000009-03</t>
+          <t>000009-08</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Lavado Automático Norte</t>
+          <t>Copec Pronto Baños</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>000009-04</t>
+          <t>000009-11</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Lavado Automático Sur</t>
+          <t>Copec Pronto Tienda</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
@@ -1087,12 +1087,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>000009-01</t>
+          <t>000009-05</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Oficina Admin.</t>
+          <t>Copec Riego</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
@@ -1105,17 +1105,17 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>000008-08</t>
+          <t>000009-02</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Alicura</t>
+          <t>Estanque Reutilización</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr"/>
@@ -1128,17 +1128,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>000008-11</t>
+          <t>000009-03</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>CE Valle Hermoso</t>
+          <t>Lavado Automático Norte</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr"/>
@@ -1151,17 +1151,17 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>000008-03</t>
+          <t>000009-04</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Carlos Fernandez P.</t>
+          <t>Lavado Automático Sur</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr"/>
@@ -1174,17 +1174,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>000008-02</t>
+          <t>000009-01</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Eduardo de la Barra</t>
+          <t>Oficina Admin.</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>000008-07</t>
+          <t>000008-08</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Erasmo Escala</t>
+          <t>Alicura</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>000008-09</t>
+          <t>000008-11</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Juan Bautista Pasten</t>
+          <t>CE Valle Hermoso</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
@@ -1248,12 +1248,12 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>000008-14</t>
+          <t>000008-03</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Juan Pablo II</t>
+          <t>Carlos Fernandez P.</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr"/>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>000008-01</t>
+          <t>000008-02</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Lic. Antonio Hermida F</t>
+          <t>Eduardo de la Barra</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>000008-13</t>
+          <t>000008-07</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Likankura</t>
+          <t>Erasmo Escala</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr"/>
@@ -1317,12 +1317,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>000008-06</t>
+          <t>000008-09</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Luis Arrieta Caña</t>
+          <t>Juan Bautista Pasten</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
@@ -1340,12 +1340,12 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>000008-10</t>
+          <t>000008-14</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Matilde Huici Navas</t>
+          <t>Juan Pablo II</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr"/>
@@ -1363,12 +1363,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>000008-05</t>
+          <t>000008-01</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Santa Maria</t>
+          <t>Lic. Antonio Hermida F</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
@@ -1386,12 +1386,12 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>000008-04</t>
+          <t>000008-13</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Tobalaba</t>
+          <t>Likankura</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr"/>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>000008-12</t>
+          <t>000008-06</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Unión Nacional Árabe</t>
+          <t>Luis Arrieta Caña</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
@@ -1427,17 +1427,17 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Club Providencia</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>000031-01</t>
+          <t>000008-10</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Matriz Fitness</t>
+          <t>Matilde Huici Navas</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr"/>
@@ -1450,17 +1450,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Club Providencia</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>000031-02</t>
+          <t>000008-05</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Matriz Piscina</t>
+          <t>Santa Maria</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr"/>
@@ -1473,17 +1473,17 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>000012-11</t>
+          <t>000008-04</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Quilicura Camarines</t>
+          <t>Tobalaba</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr"/>
@@ -1496,17 +1496,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>000012-09</t>
+          <t>000008-12</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Quilicura Casino</t>
+          <t>Unión Nacional Árabe</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr"/>
@@ -1519,17 +1519,17 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>000012-07</t>
+          <t>000031-01</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Quilicura Dercomaq</t>
+          <t>Matriz Fitness</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr"/>
@@ -1542,17 +1542,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>000012-12</t>
+          <t>000031-02</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Quilicura Edificio JCB</t>
+          <t>Matriz Piscina</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr"/>
@@ -1570,12 +1570,12 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>000012-08</t>
+          <t>000012-11</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Quilicura Lav. de Maquinas</t>
+          <t>Quilicura Camarines</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr"/>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>000012-06</t>
+          <t>000012-09</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Quilicura Matriz Principal</t>
+          <t>Quilicura Casino</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr"/>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>000012-10</t>
+          <t>000012-07</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Quilicura Proderco</t>
+          <t>Quilicura Dercomaq</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr"/>
@@ -1634,17 +1634,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Fundo Zapallar</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>000027-02</t>
+          <t>000012-12</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Estanque Inferior</t>
+          <t>Quilicura Edificio JCB</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr"/>
@@ -1657,17 +1657,17 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Fundo Zapallar</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>000027-06</t>
+          <t>000012-08</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Etapa N°1</t>
+          <t>Quilicura Lav. de Maquinas</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr"/>
@@ -1680,17 +1680,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Fundo Zapallar</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>000027-04</t>
+          <t>000012-06</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Etapa N°1 al 4</t>
+          <t>Quilicura Matriz Principal</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr"/>
@@ -1703,17 +1703,17 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Fundo Zapallar</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>000027-07</t>
+          <t>000012-10</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Etapa N°2</t>
+          <t>Quilicura Proderco</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr"/>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>000027-08</t>
+          <t>000027-02</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Etapa N°3</t>
+          <t>Estanque Inferior</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr"/>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>000027-03</t>
+          <t>000027-06</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Etapa N°5</t>
+          <t>Etapa N°1</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr"/>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>000027-01</t>
+          <t>000027-04</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Matriz ESVAL</t>
+          <t>Etapa N°1 al 4</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
@@ -1800,12 +1800,12 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>000027-09</t>
+          <t>000027-07</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Riego Llenado de Estanque ESVAL</t>
+          <t>Etapa N°2</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
@@ -1818,17 +1818,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>La Florida</t>
+          <t>Fundo Zapallar</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>000028-01</t>
+          <t>000027-08</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Liceo Alto Cordillera</t>
+          <t>Etapa N°3</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr"/>
@@ -1841,17 +1841,17 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>La Reina</t>
+          <t>Fundo Zapallar</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>000024-01</t>
+          <t>000027-03</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Eugenio María De Hostos</t>
+          <t>Etapa N°5</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr"/>
@@ -1864,17 +1864,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Las Condes</t>
+          <t>Fundo Zapallar</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>000022-00</t>
+          <t>000027-01</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Alexander Fleming</t>
+          <t>Matriz ESVAL</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr"/>
@@ -1887,17 +1887,17 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Lo valledor</t>
+          <t>Fundo Zapallar</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>000002-03</t>
+          <t>000027-09</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Lo Valledor - Barrio Norte</t>
+          <t>Riego Llenado de Estanque ESVAL</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
@@ -1910,17 +1910,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Lo valledor</t>
+          <t>La Florida</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>000002-01</t>
+          <t>000028-01</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Lo Valledor - P1</t>
+          <t>Liceo Alto Cordillera</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr"/>
@@ -1933,17 +1933,17 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>Nido de Aguilas</t>
+          <t>La Reina</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>000007-04</t>
+          <t>000024-01</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Elementary</t>
+          <t>Eugenio María De Hostos</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
@@ -1956,17 +1956,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Nido de Aguilas</t>
+          <t>Las Condes</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>000007-01</t>
+          <t>000022-00</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Estanque B</t>
+          <t>Alexander Fleming</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr"/>
@@ -1979,17 +1979,17 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Nido de Aguilas</t>
+          <t>Lo valledor</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>000007-07</t>
+          <t>000002-03</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Estanque C</t>
+          <t>Lo Valledor - Barrio Norte</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
@@ -2002,17 +2002,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Nido de Aguilas</t>
+          <t>Lo valledor</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>000007-03</t>
+          <t>000002-01</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Nido High School</t>
+          <t>Lo Valledor - P1</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr"/>
@@ -2030,12 +2030,12 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>000007-05</t>
+          <t>000007-04</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Nido Piscina</t>
+          <t>Elementary</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr"/>
@@ -2053,12 +2053,12 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>000007-06</t>
+          <t>000007-01</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Nido Pozo Profundo</t>
+          <t>Estanque B</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr"/>
@@ -2076,12 +2076,12 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>000007-02</t>
+          <t>000007-07</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Teatro</t>
+          <t>Estanque C</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr"/>
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>Nido de Aguilas</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>000025-02</t>
+          <t>000007-03</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Abastecimiento Sur Terminal</t>
+          <t>Nido High School</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr"/>
@@ -2117,17 +2117,17 @@
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>Nido de Aguilas</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>000025-34</t>
+          <t>000007-05</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Alimentación Baños</t>
+          <t>Nido Piscina</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr"/>
@@ -2140,17 +2140,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>Nido de Aguilas</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>000025-12</t>
+          <t>000007-06</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Anillo Plaza</t>
+          <t>Nido Pozo Profundo</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr"/>
@@ -2163,17 +2163,17 @@
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>Nido de Aguilas</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>000025-04</t>
+          <t>000007-02</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Baños Públicos</t>
+          <t>Teatro</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr"/>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>000025-38</t>
+          <t>000025-02</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>CUR Anillo Norte</t>
+          <t>Abastecimiento Sur Terminal</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr"/>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>000025-37</t>
+          <t>000025-34</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>CUR Anillo Sur</t>
+          <t>Alimentación Baños</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr"/>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>000025-27</t>
+          <t>000025-12</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Distrito de lujo DL</t>
+          <t>Anillo Plaza</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr"/>
@@ -2260,12 +2260,12 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>000025-01</t>
+          <t>000025-04</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Estanque Norte Locales Mall</t>
+          <t>Baños Públicos</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr"/>
@@ -2283,12 +2283,12 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>000025-21</t>
+          <t>000025-38</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Impulsión Anden 3-4 Locales Gast.</t>
+          <t>CUR Anillo Norte</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr"/>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>000025-20</t>
+          <t>000025-37</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Impulsión Anden 3-4 Matriz Principal</t>
+          <t>CUR Anillo Sur</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr"/>
@@ -2329,12 +2329,12 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>000025-29</t>
+          <t>000025-27</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Impulsión Anden 3-4 Restaurante</t>
+          <t>Distrito de lujo DL</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr"/>
@@ -2352,12 +2352,12 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>000025-10</t>
+          <t>000025-01</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Impulsión Ripley</t>
+          <t>Estanque Norte Locales Mall</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr"/>
@@ -2375,12 +2375,12 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>000025-23</t>
+          <t>000025-21</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Llenado Pileta</t>
+          <t>Impulsión Anden 3-4 Locales Gast.</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr"/>
@@ -2398,12 +2398,12 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>000025-24</t>
+          <t>000025-20</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Llenado Pileta Cascada</t>
+          <t>Impulsión Anden 3-4 Matriz Principal</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr"/>
@@ -2421,12 +2421,12 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>000025-32</t>
+          <t>000025-29</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Matriz Pasillo Tecnico Boulevard</t>
+          <t>Impulsión Anden 3-4 Restaurante</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr"/>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>000025-13</t>
+          <t>000025-10</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Matriz Principal</t>
+          <t>Impulsión Ripley</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr"/>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>000025-35</t>
+          <t>000025-23</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>PAK BAZAR GOURMET</t>
+          <t>Llenado Pileta</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr"/>
@@ -2490,12 +2490,12 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>000025-36</t>
+          <t>000025-24</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>PAK DL KENNEDY</t>
+          <t>Llenado Pileta Cascada</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr"/>
@@ -2513,12 +2513,12 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>000025-07</t>
+          <t>000025-32</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>Matriz Pasillo Tecnico Boulevard</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr"/>
@@ -2536,12 +2536,12 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>000025-08</t>
+          <t>000025-13</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Placa Bancaria</t>
+          <t>Matriz Principal</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr"/>
@@ -2559,12 +2559,12 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>000025-19</t>
+          <t>000025-35</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Sala de Bomba Estanque Sur</t>
+          <t>PAK BAZAR GOURMET</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr"/>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>000025-22</t>
+          <t>000025-36</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Sala de Bomba Sandia Antigua</t>
+          <t>PAK DL KENNEDY</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr"/>
@@ -2605,12 +2605,12 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>000025-28</t>
+          <t>000025-07</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Sala de Bomba Sandia Nueva</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr"/>
@@ -2628,12 +2628,12 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>000025-33</t>
+          <t>000025-08</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Salida de emergencia pasillo 1 ARROW</t>
+          <t>Placa Bancaria</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr"/>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>000025-17</t>
+          <t>000025-19</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>San Ignacio 300</t>
+          <t>Sala de Bomba Estanque Sur</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr"/>
@@ -2674,12 +2674,12 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>000025-18</t>
+          <t>000025-22</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>San Ignacio 500</t>
+          <t>Sala de Bomba Sandia Antigua</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr"/>
@@ -2692,17 +2692,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>000006-02</t>
+          <t>000025-28</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Carmela Carvajal</t>
+          <t>Sala de Bomba Sandia Nueva</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr"/>
@@ -2715,17 +2715,17 @@
       </c>
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>000006-04</t>
+          <t>000025-33</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Liceo 7 Luisa Saavedra</t>
+          <t>Salida de emergencia pasillo 1 ARROW</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
@@ -2738,17 +2738,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>000006-05</t>
+          <t>000025-17</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>Liceo Juan Pablo Duarte</t>
+          <t>San Ignacio 300</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr"/>
@@ -2761,17 +2761,17 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>000006-01</t>
+          <t>000025-18</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Liceo Lastarria</t>
+          <t>San Ignacio 500</t>
         </is>
       </c>
       <c r="E98" s="6" t="inlineStr"/>
@@ -2784,17 +2784,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>000017-08</t>
+          <t>000006-02</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Cumbre de cóndores Ote.</t>
+          <t>Carmela Carvajal</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr"/>
@@ -2807,17 +2807,17 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>000017-07</t>
+          <t>000006-04</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Cumbre de cóndores pte.</t>
+          <t>Liceo 7 Luisa Saavedra</t>
         </is>
       </c>
       <c r="E100" s="6" t="inlineStr"/>
@@ -2830,17 +2830,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>000017-04</t>
+          <t>000006-05</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Esc. Lo Velásquez</t>
+          <t>Liceo Juan Pablo Duarte</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr"/>
@@ -2853,17 +2853,17 @@
       </c>
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>000017-05</t>
+          <t>000006-01</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Gimnasio</t>
+          <t>Liceo Lastarria</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr"/>
@@ -2881,29 +2881,121 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>000017-06</t>
+          <t>000017-08</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Piscina Municipal</t>
+          <t>Cumbre de cóndores Ote.</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr"/>
       <c r="F103" s="6" t="inlineStr"/>
       <c r="G103" s="7" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>000017-07</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>Cumbre de cóndores pte.</t>
+        </is>
+      </c>
+      <c r="E104" s="6" t="inlineStr"/>
+      <c r="F104" s="6" t="inlineStr"/>
+      <c r="G104" s="7" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>000017-04</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Esc. Lo Velásquez</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr"/>
+      <c r="F105" s="6" t="inlineStr"/>
+      <c r="G105" s="7" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>000017-05</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>Gimnasio</t>
+        </is>
+      </c>
+      <c r="E106" s="6" t="inlineStr"/>
+      <c r="F106" s="6" t="inlineStr"/>
+      <c r="G106" s="7" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>000017-06</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Piscina Municipal</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr"/>
+      <c r="F107" s="6" t="inlineStr"/>
+      <c r="G107" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G103"/>
+  <autoFilter ref="A4:G107"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Monitoreo" error="Elija una opción de la lista (o borre la celda)." promptTitle="Monitoreo" prompt="Seleccione un valor para Monitoreo o déjelo en blanco" type="list">
+    <dataValidation sqref="E5:E107" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Monitoreo" error="Elija una opción de la lista (o borre la celda)." promptTitle="Monitoreo" prompt="Seleccione un valor para Monitoreo o déjelo en blanco" type="list">
       <formula1>"Sí,No,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Control" error="Elija una opción de la lista (o borre la celda)." promptTitle="Control" prompt="Seleccione un valor para Control o déjelo en blanco" type="list">
+    <dataValidation sqref="F5:F107" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Control" error="Elija una opción de la lista (o borre la celda)." promptTitle="Control" prompt="Seleccione un valor para Control o déjelo en blanco" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2919,7 +3011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2937,7 +3029,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 16:59 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 17:04 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -2968,7 +3060,7 @@
         <v>26</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.2626262626262627</v>
+        <v>0.2524271844660194</v>
       </c>
     </row>
     <row r="6">
@@ -2981,7 +3073,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>0.1414141414141414</v>
+        <v>0.1359223300970874</v>
       </c>
     </row>
     <row r="7">
@@ -2994,7 +3086,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1067961165048544</v>
       </c>
     </row>
     <row r="8">
@@ -3007,7 +3099,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>0.08080808080808081</v>
+        <v>0.07766990291262135</v>
       </c>
     </row>
     <row r="9">
@@ -3020,7 +3112,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>0.0707070707070707</v>
+        <v>0.06796116504854369</v>
       </c>
     </row>
     <row r="10">
@@ -3033,7 +3125,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>0.0707070707070707</v>
+        <v>0.06796116504854369</v>
       </c>
     </row>
     <row r="11">
@@ -3046,7 +3138,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.0505050505050505</v>
+        <v>0.04854368932038835</v>
       </c>
     </row>
     <row r="12">
@@ -3059,7 +3151,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>0.0505050505050505</v>
+        <v>0.04854368932038835</v>
       </c>
     </row>
     <row r="13">
@@ -3072,102 +3164,115 @@
         <v>5</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>0.0505050505050505</v>
+        <v>0.04854368932038835</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>BUPA Antofagasta</t>
         </is>
       </c>
       <c r="B14" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>0.04040404040404041</v>
+        <v>0.03883495145631068</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Club Providencia</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>0.0202020202020202</v>
+        <v>0.03883495145631068</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Lo valledor</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="B16" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>0.0202020202020202</v>
+        <v>0.01941747572815534</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>La Florida</t>
+          <t>Lo valledor</t>
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>0.0101010101010101</v>
+        <v>0.01941747572815534</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>La Reina</t>
+          <t>La Florida</t>
         </is>
       </c>
       <c r="B18" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>0.0101010101010101</v>
+        <v>0.009708737864077669</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Las Condes</t>
+          <t>La Reina</t>
         </is>
       </c>
       <c r="B19" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>0.0101010101010101</v>
+        <v>0.009708737864077669</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>0.009708737864077669</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n">
-        <v>99</v>
-      </c>
-      <c r="C20" s="18" t="n">
+      <c r="B21" s="17" t="n">
+        <v>103</v>
+      </c>
+      <c r="C21" s="18" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C19"/>
+  <autoFilter ref="A4:C20"/>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -3217,7 +3322,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>26/08/2026 16:59 hora Chile</t>
+          <t>26/08/2026 17:04 hora Chile</t>
         </is>
       </c>
     </row>
@@ -3229,7 +3334,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>103</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3358,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>Empresas y nodos excluidos (WES, Ejército, Gendarmería, BUPA pendiente de instalación, Corporación Puente Alto, MOP, Lo Boza, TML, MADECO, IDs en exclusiones_reportes.py y registro_puntos_deshabilitados.txt).</t>
+          <t>Empresas y nodos excluidos (WES, Ejército, Gendarmería, BUPA 01-06 pendiente de instalación, Corporación Puente Alto, MOP, Lo Boza, TML, MADECO, IDs en exclusiones_reportes.py y registro_puntos_deshabilitados.txt). Sí incluye BUPA Antofagasta (000029-07..10).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the equipment Excel with 28 Parque Arauco points.
Adds Impulsión Falabella and Matriz A.A; the workbook now has 105 vigentes.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Cómo usar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equipos vigentes'!$A$4:$G$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equipos vigentes'!$A$4:$G$109</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Equipos vigentes'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen por cliente'!$A$4:$C$20</definedName>
   </definedNames>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 26/08/2026 17:04 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
+          <t>Equipos vigentes al 26/08/2026 17:10 (hora Chile). Mismo universo que el reporte matinal de puntos en cero (API WES + exclusiones vigentes). Complete las columnas Monitoreo y Control.</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>000025-10</t>
+          <t>000025-09</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Impulsión Ripley</t>
+          <t>Impulsión Falabella</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr"/>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>000025-23</t>
+          <t>000025-10</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Llenado Pileta</t>
+          <t>Impulsión Ripley</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr"/>
@@ -2490,12 +2490,12 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>000025-24</t>
+          <t>000025-23</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Llenado Pileta Cascada</t>
+          <t>Llenado Pileta</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr"/>
@@ -2513,12 +2513,12 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>000025-32</t>
+          <t>000025-24</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Matriz Pasillo Tecnico Boulevard</t>
+          <t>Llenado Pileta Cascada</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr"/>
@@ -2536,12 +2536,12 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>000025-13</t>
+          <t>000025-30</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Matriz Principal</t>
+          <t>Matriz A.A</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr"/>
@@ -2559,12 +2559,12 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>000025-35</t>
+          <t>000025-32</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>PAK BAZAR GOURMET</t>
+          <t>Matriz Pasillo Tecnico Boulevard</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr"/>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>000025-36</t>
+          <t>000025-13</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>PAK DL KENNEDY</t>
+          <t>Matriz Principal</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr"/>
@@ -2605,12 +2605,12 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>000025-07</t>
+          <t>000025-35</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>PAK BAZAR GOURMET</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr"/>
@@ -2628,12 +2628,12 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>000025-08</t>
+          <t>000025-36</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Placa Bancaria</t>
+          <t>PAK DL KENNEDY</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr"/>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>000025-19</t>
+          <t>000025-07</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Sala de Bomba Estanque Sur</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr"/>
@@ -2674,12 +2674,12 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>000025-22</t>
+          <t>000025-08</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Sala de Bomba Sandia Antigua</t>
+          <t>Placa Bancaria</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr"/>
@@ -2697,12 +2697,12 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>000025-28</t>
+          <t>000025-19</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Sala de Bomba Sandia Nueva</t>
+          <t>Sala de Bomba Estanque Sur</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr"/>
@@ -2720,12 +2720,12 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>000025-33</t>
+          <t>000025-22</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Salida de emergencia pasillo 1 ARROW</t>
+          <t>Sala de Bomba Sandia Antigua</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
@@ -2743,12 +2743,12 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>000025-17</t>
+          <t>000025-28</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>San Ignacio 300</t>
+          <t>Sala de Bomba Sandia Nueva</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr"/>
@@ -2766,12 +2766,12 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>000025-18</t>
+          <t>000025-33</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>San Ignacio 500</t>
+          <t>Salida de emergencia pasillo 1 ARROW</t>
         </is>
       </c>
       <c r="E98" s="6" t="inlineStr"/>
@@ -2784,17 +2784,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>000006-02</t>
+          <t>000025-17</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Carmela Carvajal</t>
+          <t>San Ignacio 300</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr"/>
@@ -2807,17 +2807,17 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>Providencia</t>
+          <t>Parque Arauco</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>000006-04</t>
+          <t>000025-18</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Liceo 7 Luisa Saavedra</t>
+          <t>San Ignacio 500</t>
         </is>
       </c>
       <c r="E100" s="6" t="inlineStr"/>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>000006-05</t>
+          <t>000006-02</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Liceo Juan Pablo Duarte</t>
+          <t>Carmela Carvajal</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr"/>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>000006-01</t>
+          <t>000006-04</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Liceo Lastarria</t>
+          <t>Liceo 7 Luisa Saavedra</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr"/>
@@ -2876,17 +2876,17 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>000017-08</t>
+          <t>000006-05</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Cumbre de cóndores Ote.</t>
+          <t>Liceo Juan Pablo Duarte</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr"/>
@@ -2899,17 +2899,17 @@
       </c>
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>Providencia</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>000017-07</t>
+          <t>000006-01</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Cumbre de cóndores pte.</t>
+          <t>Liceo Lastarria</t>
         </is>
       </c>
       <c r="E104" s="6" t="inlineStr"/>
@@ -2927,12 +2927,12 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>000017-04</t>
+          <t>000017-08</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>Esc. Lo Velásquez</t>
+          <t>Cumbre de cóndores Ote.</t>
         </is>
       </c>
       <c r="E105" s="6" t="inlineStr"/>
@@ -2950,12 +2950,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>000017-05</t>
+          <t>000017-07</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Gimnasio</t>
+          <t>Cumbre de cóndores pte.</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr"/>
@@ -2973,29 +2973,75 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>000017-06</t>
+          <t>000017-04</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Piscina Municipal</t>
+          <t>Esc. Lo Velásquez</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr"/>
       <c r="F107" s="6" t="inlineStr"/>
       <c r="G107" s="7" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" s="8" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>000017-05</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>Gimnasio</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr"/>
+      <c r="F108" s="6" t="inlineStr"/>
+      <c r="G108" s="7" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>000017-06</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>Piscina Municipal</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr"/>
+      <c r="F109" s="6" t="inlineStr"/>
+      <c r="G109" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G107"/>
+  <autoFilter ref="A4:G109"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E107" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Monitoreo" error="Elija una opción de la lista (o borre la celda)." promptTitle="Monitoreo" prompt="Seleccione un valor para Monitoreo o déjelo en blanco" type="list">
+    <dataValidation sqref="E5:E109" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Monitoreo" error="Elija una opción de la lista (o borre la celda)." promptTitle="Monitoreo" prompt="Seleccione un valor para Monitoreo o déjelo en blanco" type="list">
       <formula1>"Sí,No,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F107" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Control" error="Elija una opción de la lista (o borre la celda)." promptTitle="Control" prompt="Seleccione un valor para Control o déjelo en blanco" type="list">
+    <dataValidation sqref="F5:F109" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Control" error="Elija una opción de la lista (o borre la celda)." promptTitle="Control" prompt="Seleccione un valor para Control o déjelo en blanco" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3029,7 +3075,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 17:04 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 17:10 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -3057,10 +3103,10 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.2524271844660194</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -3073,7 +3119,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>0.1359223300970874</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -3086,7 +3132,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>0.1067961165048544</v>
+        <v>0.1047619047619048</v>
       </c>
     </row>
     <row r="8">
@@ -3099,7 +3145,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>0.07766990291262135</v>
+        <v>0.0761904761904762</v>
       </c>
     </row>
     <row r="9">
@@ -3112,7 +3158,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>0.06796116504854369</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -3125,7 +3171,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>0.06796116504854369</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="11">
@@ -3138,7 +3184,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.04854368932038835</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="12">
@@ -3151,7 +3197,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>0.04854368932038835</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="13">
@@ -3164,7 +3210,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>0.04854368932038835</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="14">
@@ -3177,7 +3223,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>0.03883495145631068</v>
+        <v>0.0380952380952381</v>
       </c>
     </row>
     <row r="15">
@@ -3190,7 +3236,7 @@
         <v>4</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>0.03883495145631068</v>
+        <v>0.0380952380952381</v>
       </c>
     </row>
     <row r="16">
@@ -3203,7 +3249,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>0.01941747572815534</v>
+        <v>0.01904761904761905</v>
       </c>
     </row>
     <row r="17">
@@ -3216,7 +3262,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>0.01941747572815534</v>
+        <v>0.01904761904761905</v>
       </c>
     </row>
     <row r="18">
@@ -3229,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>0.009708737864077669</v>
+        <v>0.009523809523809525</v>
       </c>
     </row>
     <row r="19">
@@ -3242,7 +3288,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>0.009708737864077669</v>
+        <v>0.009523809523809525</v>
       </c>
     </row>
     <row r="20">
@@ -3255,7 +3301,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>0.009708737864077669</v>
+        <v>0.009523809523809525</v>
       </c>
     </row>
     <row r="21">
@@ -3265,7 +3311,7 @@
         </is>
       </c>
       <c r="B21" s="17" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C21" s="18" t="n">
         <v>1</v>
@@ -3322,7 +3368,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>26/08/2026 17:04 hora Chile</t>
+          <t>26/08/2026 17:10 hora Chile</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3380,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>105</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the two confirmed COPEC cabinets in the equipment Excel.
Four wash points share one 4-plate cabinet; matriz, riego and estanque share a 3-plate cabinet. Other rows stay for the user to complete.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -578,7 +578,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 26/08/2026 17:30 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Monitoreo y Control: Sí/No.</t>
+          <t>Equipos vigentes al 28/08/2026 11:28 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,11 @@
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr">
         <is>
@@ -688,7 +692,11 @@
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -722,7 +730,11 @@
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -756,7 +768,11 @@
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -790,7 +806,11 @@
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="7" t="inlineStr">
         <is>
@@ -824,7 +844,11 @@
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr">
         <is>
@@ -858,7 +882,11 @@
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr">
         <is>
@@ -892,7 +920,11 @@
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="7" t="inlineStr">
         <is>
@@ -926,7 +958,11 @@
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -960,7 +996,11 @@
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="7" t="inlineStr">
         <is>
@@ -994,7 +1034,11 @@
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr">
         <is>
@@ -1028,7 +1072,11 @@
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="7" t="inlineStr">
         <is>
@@ -1062,7 +1110,11 @@
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="7" t="inlineStr">
         <is>
@@ -1096,7 +1148,11 @@
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="7" t="inlineStr">
         <is>
@@ -1130,7 +1186,11 @@
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="7" t="inlineStr">
         <is>
@@ -1163,9 +1223,21 @@
           <t>Copec Lavado Auto servicio Norte</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Lavados</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>4 placas</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>000009-03 Lavado Automático Norte; 000009-04 Lavado Automático Sur; 000009-09 Copec Lavado Auto servicio Norte; 000009-10 Copec Lavado Auto servicio Sur</t>
+        </is>
+      </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1197,9 +1269,21 @@
           <t>Copec Lavado Auto servicio Sur</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Lavados</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>4 placas</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>000009-03 Lavado Automático Norte; 000009-04 Lavado Automático Sur; 000009-09 Copec Lavado Auto servicio Norte; 000009-10 Copec Lavado Auto servicio Sur</t>
+        </is>
+      </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1231,9 +1315,21 @@
           <t>Copec Matriz Principal</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Matriz / riego / estanque</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>000009-02 Estanque Reutilización; 000009-05 Copec Riego; 000009-06 Copec Matriz Principal</t>
+        </is>
+      </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1266,7 +1362,11 @@
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr"/>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G23" s="6" t="inlineStr"/>
       <c r="H23" s="7" t="inlineStr">
         <is>
@@ -1300,7 +1400,11 @@
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="7" t="inlineStr">
         <is>
@@ -1333,9 +1437,21 @@
           <t>Copec Riego</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Matriz / riego / estanque</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>000009-02 Estanque Reutilización; 000009-05 Copec Riego; 000009-06 Copec Matriz Principal</t>
+        </is>
+      </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1367,9 +1483,21 @@
           <t>Estanque Reutilización</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Matriz / riego / estanque</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>000009-02 Estanque Reutilización; 000009-05 Copec Riego; 000009-06 Copec Matriz Principal</t>
+        </is>
+      </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1401,9 +1529,21 @@
           <t>Lavado Automático Norte</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="7" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Lavados</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>4 placas</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>000009-03 Lavado Automático Norte; 000009-04 Lavado Automático Sur; 000009-09 Copec Lavado Auto servicio Norte; 000009-10 Copec Lavado Auto servicio Sur</t>
+        </is>
+      </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1435,9 +1575,21 @@
           <t>Lavado Automático Sur</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Lavados</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>4 placas</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>000009-03 Lavado Automático Norte; 000009-04 Lavado Automático Sur; 000009-09 Copec Lavado Auto servicio Norte; 000009-10 Copec Lavado Auto servicio Sur</t>
+        </is>
+      </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1470,7 +1622,11 @@
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="7" t="inlineStr"/>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G29" s="6" t="inlineStr"/>
       <c r="H29" s="7" t="inlineStr">
         <is>
@@ -1504,7 +1660,11 @@
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="7" t="inlineStr"/>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G30" s="6" t="inlineStr"/>
       <c r="H30" s="7" t="inlineStr">
         <is>
@@ -1538,7 +1698,11 @@
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
-      <c r="F31" s="7" t="inlineStr"/>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G31" s="6" t="inlineStr"/>
       <c r="H31" s="7" t="inlineStr">
         <is>
@@ -1572,7 +1736,11 @@
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="7" t="inlineStr"/>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G32" s="6" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr">
         <is>
@@ -1606,7 +1774,11 @@
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="7" t="inlineStr"/>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G33" s="6" t="inlineStr"/>
       <c r="H33" s="7" t="inlineStr">
         <is>
@@ -1640,7 +1812,11 @@
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="7" t="inlineStr"/>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G34" s="6" t="inlineStr"/>
       <c r="H34" s="7" t="inlineStr">
         <is>
@@ -1674,7 +1850,11 @@
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
-      <c r="F35" s="7" t="inlineStr"/>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G35" s="6" t="inlineStr"/>
       <c r="H35" s="7" t="inlineStr">
         <is>
@@ -1708,7 +1888,11 @@
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="7" t="inlineStr"/>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G36" s="6" t="inlineStr"/>
       <c r="H36" s="7" t="inlineStr">
         <is>
@@ -1742,7 +1926,11 @@
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
-      <c r="F37" s="7" t="inlineStr"/>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G37" s="6" t="inlineStr"/>
       <c r="H37" s="7" t="inlineStr">
         <is>
@@ -1776,7 +1964,11 @@
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="7" t="inlineStr"/>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G38" s="6" t="inlineStr"/>
       <c r="H38" s="7" t="inlineStr">
         <is>
@@ -1810,7 +2002,11 @@
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="7" t="inlineStr"/>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G39" s="6" t="inlineStr"/>
       <c r="H39" s="7" t="inlineStr">
         <is>
@@ -1844,7 +2040,11 @@
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr"/>
-      <c r="F40" s="7" t="inlineStr"/>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G40" s="6" t="inlineStr"/>
       <c r="H40" s="7" t="inlineStr">
         <is>
@@ -1878,7 +2078,11 @@
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr"/>
-      <c r="F41" s="7" t="inlineStr"/>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G41" s="6" t="inlineStr"/>
       <c r="H41" s="7" t="inlineStr">
         <is>
@@ -1912,7 +2116,11 @@
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr"/>
-      <c r="F42" s="7" t="inlineStr"/>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G42" s="6" t="inlineStr"/>
       <c r="H42" s="7" t="inlineStr">
         <is>
@@ -1946,7 +2154,11 @@
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr"/>
-      <c r="F43" s="7" t="inlineStr"/>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G43" s="6" t="inlineStr"/>
       <c r="H43" s="7" t="inlineStr">
         <is>
@@ -1980,7 +2192,11 @@
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr"/>
-      <c r="F44" s="7" t="inlineStr"/>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G44" s="6" t="inlineStr"/>
       <c r="H44" s="7" t="inlineStr">
         <is>
@@ -2014,7 +2230,11 @@
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="7" t="inlineStr"/>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G45" s="6" t="inlineStr"/>
       <c r="H45" s="7" t="inlineStr">
         <is>
@@ -2048,7 +2268,11 @@
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr"/>
-      <c r="F46" s="7" t="inlineStr"/>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G46" s="6" t="inlineStr"/>
       <c r="H46" s="7" t="inlineStr">
         <is>
@@ -2082,7 +2306,11 @@
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr"/>
-      <c r="F47" s="7" t="inlineStr"/>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G47" s="6" t="inlineStr"/>
       <c r="H47" s="7" t="inlineStr">
         <is>
@@ -2116,7 +2344,11 @@
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr"/>
-      <c r="F48" s="7" t="inlineStr"/>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G48" s="6" t="inlineStr"/>
       <c r="H48" s="7" t="inlineStr">
         <is>
@@ -2150,7 +2382,11 @@
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr"/>
-      <c r="F49" s="7" t="inlineStr"/>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G49" s="6" t="inlineStr"/>
       <c r="H49" s="7" t="inlineStr">
         <is>
@@ -2184,7 +2420,11 @@
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr"/>
-      <c r="F50" s="7" t="inlineStr"/>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G50" s="6" t="inlineStr"/>
       <c r="H50" s="7" t="inlineStr">
         <is>
@@ -2218,7 +2458,11 @@
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr"/>
-      <c r="F51" s="7" t="inlineStr"/>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G51" s="6" t="inlineStr"/>
       <c r="H51" s="7" t="inlineStr">
         <is>
@@ -2252,7 +2496,11 @@
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr"/>
-      <c r="F52" s="7" t="inlineStr"/>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G52" s="6" t="inlineStr"/>
       <c r="H52" s="7" t="inlineStr">
         <is>
@@ -2286,7 +2534,11 @@
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr"/>
-      <c r="F53" s="7" t="inlineStr"/>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G53" s="6" t="inlineStr"/>
       <c r="H53" s="7" t="inlineStr">
         <is>
@@ -2320,7 +2572,11 @@
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr"/>
-      <c r="F54" s="7" t="inlineStr"/>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G54" s="6" t="inlineStr"/>
       <c r="H54" s="7" t="inlineStr">
         <is>
@@ -2354,7 +2610,11 @@
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
-      <c r="F55" s="7" t="inlineStr"/>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G55" s="6" t="inlineStr"/>
       <c r="H55" s="7" t="inlineStr">
         <is>
@@ -2388,7 +2648,11 @@
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
-      <c r="F56" s="7" t="inlineStr"/>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G56" s="6" t="inlineStr"/>
       <c r="H56" s="7" t="inlineStr">
         <is>
@@ -2422,7 +2686,11 @@
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr"/>
-      <c r="F57" s="7" t="inlineStr"/>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G57" s="6" t="inlineStr"/>
       <c r="H57" s="7" t="inlineStr">
         <is>
@@ -2456,7 +2724,11 @@
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr"/>
-      <c r="F58" s="7" t="inlineStr"/>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G58" s="6" t="inlineStr"/>
       <c r="H58" s="7" t="inlineStr">
         <is>
@@ -2490,7 +2762,11 @@
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr"/>
-      <c r="F59" s="7" t="inlineStr"/>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G59" s="6" t="inlineStr"/>
       <c r="H59" s="7" t="inlineStr">
         <is>
@@ -2524,7 +2800,11 @@
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
-      <c r="F60" s="7" t="inlineStr"/>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G60" s="6" t="inlineStr"/>
       <c r="H60" s="7" t="inlineStr">
         <is>
@@ -2558,7 +2838,11 @@
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr"/>
-      <c r="F61" s="7" t="inlineStr"/>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G61" s="6" t="inlineStr"/>
       <c r="H61" s="7" t="inlineStr">
         <is>
@@ -2592,7 +2876,11 @@
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
-      <c r="F62" s="7" t="inlineStr"/>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G62" s="6" t="inlineStr"/>
       <c r="H62" s="7" t="inlineStr">
         <is>
@@ -2626,7 +2914,11 @@
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr"/>
-      <c r="F63" s="7" t="inlineStr"/>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G63" s="6" t="inlineStr"/>
       <c r="H63" s="7" t="inlineStr">
         <is>
@@ -2660,7 +2952,11 @@
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
-      <c r="F64" s="7" t="inlineStr"/>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G64" s="6" t="inlineStr"/>
       <c r="H64" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2990,11 @@
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr"/>
-      <c r="F65" s="7" t="inlineStr"/>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G65" s="6" t="inlineStr"/>
       <c r="H65" s="7" t="inlineStr">
         <is>
@@ -2728,7 +3028,11 @@
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr"/>
-      <c r="F66" s="7" t="inlineStr"/>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="7" t="inlineStr">
         <is>
@@ -2762,7 +3066,11 @@
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr"/>
-      <c r="F67" s="7" t="inlineStr"/>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G67" s="6" t="inlineStr"/>
       <c r="H67" s="7" t="inlineStr">
         <is>
@@ -2796,7 +3104,11 @@
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr"/>
-      <c r="F68" s="7" t="inlineStr"/>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G68" s="6" t="inlineStr"/>
       <c r="H68" s="7" t="inlineStr">
         <is>
@@ -2830,7 +3142,11 @@
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr"/>
-      <c r="F69" s="7" t="inlineStr"/>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G69" s="6" t="inlineStr"/>
       <c r="H69" s="7" t="inlineStr">
         <is>
@@ -2864,7 +3180,11 @@
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr"/>
-      <c r="F70" s="7" t="inlineStr"/>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G70" s="6" t="inlineStr"/>
       <c r="H70" s="7" t="inlineStr">
         <is>
@@ -2898,7 +3218,11 @@
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr"/>
-      <c r="F71" s="7" t="inlineStr"/>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G71" s="6" t="inlineStr"/>
       <c r="H71" s="7" t="inlineStr">
         <is>
@@ -2932,7 +3256,11 @@
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr"/>
-      <c r="F72" s="7" t="inlineStr"/>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="7" t="inlineStr">
         <is>
@@ -2966,7 +3294,11 @@
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr"/>
-      <c r="F73" s="7" t="inlineStr"/>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="7" t="inlineStr">
         <is>
@@ -3000,7 +3332,11 @@
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr"/>
-      <c r="F74" s="7" t="inlineStr"/>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G74" s="6" t="inlineStr"/>
       <c r="H74" s="7" t="inlineStr">
         <is>
@@ -3034,7 +3370,11 @@
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr"/>
-      <c r="F75" s="7" t="inlineStr"/>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="7" t="inlineStr">
         <is>
@@ -3068,7 +3408,11 @@
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="7" t="inlineStr"/>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="7" t="inlineStr">
         <is>
@@ -3102,7 +3446,11 @@
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr"/>
-      <c r="F77" s="7" t="inlineStr"/>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="7" t="inlineStr">
         <is>
@@ -3136,7 +3484,11 @@
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>2 placas</t>
+        </is>
+      </c>
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="7" t="inlineStr">
         <is>
@@ -3170,7 +3522,11 @@
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr"/>
-      <c r="F79" s="7" t="inlineStr"/>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G79" s="6" t="inlineStr"/>
       <c r="H79" s="7" t="inlineStr">
         <is>
@@ -3204,7 +3560,11 @@
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr"/>
-      <c r="F80" s="7" t="inlineStr"/>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G80" s="6" t="inlineStr"/>
       <c r="H80" s="7" t="inlineStr">
         <is>
@@ -3238,7 +3598,11 @@
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr"/>
-      <c r="F81" s="7" t="inlineStr"/>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="7" t="inlineStr">
         <is>
@@ -3272,7 +3636,11 @@
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr"/>
-      <c r="F82" s="7" t="inlineStr"/>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G82" s="6" t="inlineStr"/>
       <c r="H82" s="7" t="inlineStr">
         <is>
@@ -3306,7 +3674,11 @@
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr"/>
-      <c r="F83" s="7" t="inlineStr"/>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>3 placas</t>
+        </is>
+      </c>
       <c r="G83" s="6" t="inlineStr"/>
       <c r="H83" s="7" t="inlineStr">
         <is>
@@ -3340,7 +3712,11 @@
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr"/>
-      <c r="F84" s="7" t="inlineStr"/>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G84" s="6" t="inlineStr"/>
       <c r="H84" s="7" t="inlineStr">
         <is>
@@ -3374,7 +3750,11 @@
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr"/>
-      <c r="F85" s="7" t="inlineStr"/>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G85" s="6" t="inlineStr"/>
       <c r="H85" s="7" t="inlineStr">
         <is>
@@ -3408,7 +3788,11 @@
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr"/>
-      <c r="F86" s="7" t="inlineStr"/>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G86" s="6" t="inlineStr"/>
       <c r="H86" s="7" t="inlineStr">
         <is>
@@ -3442,7 +3826,11 @@
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr"/>
-      <c r="F87" s="7" t="inlineStr"/>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G87" s="6" t="inlineStr"/>
       <c r="H87" s="7" t="inlineStr">
         <is>
@@ -3476,7 +3864,11 @@
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr"/>
-      <c r="F88" s="7" t="inlineStr"/>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G88" s="6" t="inlineStr"/>
       <c r="H88" s="7" t="inlineStr">
         <is>
@@ -3510,7 +3902,11 @@
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr"/>
-      <c r="F89" s="7" t="inlineStr"/>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G89" s="6" t="inlineStr"/>
       <c r="H89" s="7" t="inlineStr">
         <is>
@@ -3544,7 +3940,11 @@
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr"/>
-      <c r="F90" s="7" t="inlineStr"/>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G90" s="6" t="inlineStr"/>
       <c r="H90" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3978,11 @@
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr"/>
-      <c r="F91" s="7" t="inlineStr"/>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G91" s="6" t="inlineStr"/>
       <c r="H91" s="7" t="inlineStr">
         <is>
@@ -3612,7 +4016,11 @@
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr"/>
-      <c r="F92" s="7" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G92" s="6" t="inlineStr"/>
       <c r="H92" s="7" t="inlineStr">
         <is>
@@ -3646,7 +4054,11 @@
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr"/>
-      <c r="F93" s="7" t="inlineStr"/>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G93" s="6" t="inlineStr"/>
       <c r="H93" s="7" t="inlineStr">
         <is>
@@ -3680,7 +4092,11 @@
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr"/>
-      <c r="F94" s="7" t="inlineStr"/>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G94" s="6" t="inlineStr"/>
       <c r="H94" s="7" t="inlineStr">
         <is>
@@ -3714,7 +4130,11 @@
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr"/>
-      <c r="F95" s="7" t="inlineStr"/>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G95" s="6" t="inlineStr"/>
       <c r="H95" s="7" t="inlineStr">
         <is>
@@ -3748,7 +4168,11 @@
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
-      <c r="F96" s="7" t="inlineStr"/>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G96" s="6" t="inlineStr"/>
       <c r="H96" s="7" t="inlineStr">
         <is>
@@ -3782,7 +4206,11 @@
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr"/>
-      <c r="F97" s="7" t="inlineStr"/>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G97" s="6" t="inlineStr"/>
       <c r="H97" s="7" t="inlineStr">
         <is>
@@ -3816,7 +4244,11 @@
         </is>
       </c>
       <c r="E98" s="6" t="inlineStr"/>
-      <c r="F98" s="7" t="inlineStr"/>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G98" s="6" t="inlineStr"/>
       <c r="H98" s="7" t="inlineStr">
         <is>
@@ -3850,7 +4282,11 @@
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr"/>
-      <c r="F99" s="7" t="inlineStr"/>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G99" s="6" t="inlineStr"/>
       <c r="H99" s="7" t="inlineStr">
         <is>
@@ -3884,7 +4320,11 @@
         </is>
       </c>
       <c r="E100" s="6" t="inlineStr"/>
-      <c r="F100" s="7" t="inlineStr"/>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G100" s="6" t="inlineStr"/>
       <c r="H100" s="7" t="inlineStr">
         <is>
@@ -3918,7 +4358,11 @@
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr"/>
-      <c r="F101" s="7" t="inlineStr"/>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G101" s="6" t="inlineStr"/>
       <c r="H101" s="7" t="inlineStr">
         <is>
@@ -3952,7 +4396,11 @@
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr"/>
-      <c r="F102" s="7" t="inlineStr"/>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G102" s="6" t="inlineStr"/>
       <c r="H102" s="7" t="inlineStr">
         <is>
@@ -3986,7 +4434,11 @@
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr"/>
-      <c r="F103" s="7" t="inlineStr"/>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G103" s="6" t="inlineStr"/>
       <c r="H103" s="7" t="inlineStr">
         <is>
@@ -4020,7 +4472,11 @@
         </is>
       </c>
       <c r="E104" s="6" t="inlineStr"/>
-      <c r="F104" s="7" t="inlineStr"/>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G104" s="6" t="inlineStr"/>
       <c r="H104" s="7" t="inlineStr">
         <is>
@@ -4054,7 +4510,11 @@
         </is>
       </c>
       <c r="E105" s="6" t="inlineStr"/>
-      <c r="F105" s="7" t="inlineStr"/>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G105" s="6" t="inlineStr"/>
       <c r="H105" s="7" t="inlineStr">
         <is>
@@ -4088,7 +4548,11 @@
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr"/>
-      <c r="F106" s="7" t="inlineStr"/>
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G106" s="6" t="inlineStr"/>
       <c r="H106" s="7" t="inlineStr">
         <is>
@@ -4122,7 +4586,11 @@
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr"/>
-      <c r="F107" s="7" t="inlineStr"/>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G107" s="6" t="inlineStr"/>
       <c r="H107" s="7" t="inlineStr">
         <is>
@@ -4156,7 +4624,11 @@
         </is>
       </c>
       <c r="E108" s="6" t="inlineStr"/>
-      <c r="F108" s="7" t="inlineStr"/>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G108" s="6" t="inlineStr"/>
       <c r="H108" s="7" t="inlineStr">
         <is>
@@ -4190,7 +4662,11 @@
         </is>
       </c>
       <c r="E109" s="6" t="inlineStr"/>
-      <c r="F109" s="7" t="inlineStr"/>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
       <c r="G109" s="6" t="inlineStr"/>
       <c r="H109" s="7" t="inlineStr">
         <is>
@@ -4251,7 +4727,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 26/08/2026 17:30 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 11:28 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -4544,7 +5020,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>26/08/2026 17:30 hora Chile</t>
+          <t>28/08/2026 11:28 hora Chile</t>
         </is>
       </c>
     </row>
@@ -4604,7 +5080,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Complete con el desplegable: 1 placa, 2 placas, 3 placas, 4 placas o 5 placas.</t>
+          <t>Complete con el desplegable: 1 a 5 placas. Ya vienen llenos los gabinetes confirmados (COPEC: 4 lavados; y matriz + riego + estanque).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the Excel with Costanera/Admin, Pronto, and Zapallar etapa cabinets.
All 11 COPEC nodes are now in confirmed gabinetes; Zapallar etapa 1-4 sits with etapa 5.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -578,7 +578,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 28/08/2026 11:28 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
+          <t>Equipos vigentes al 28/08/2026 11:33 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
         </is>
       </c>
     </row>
@@ -1185,13 +1185,21 @@
           <t>Copec Costanera</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Costanera / Oficina Admin.</t>
+        </is>
+      </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>000009-00 Copec Costanera; 000009-01 Oficina Admin.</t>
+        </is>
+      </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1361,13 +1369,21 @@
           <t>Copec Pronto Baños</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Pronto</t>
+        </is>
+      </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>000009-08 Copec Pronto Baños; 000009-11 Copec Pronto Tienda</t>
+        </is>
+      </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1399,13 +1415,21 @@
           <t>Copec Pronto Tienda</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Pronto</t>
+        </is>
+      </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>000009-08 Copec Pronto Baños; 000009-11 Copec Pronto Tienda</t>
+        </is>
+      </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1621,13 +1645,21 @@
           <t>Oficina Admin.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>COPEC Costanera — Costanera / Oficina Admin.</t>
+        </is>
+      </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>000009-00 Copec Costanera; 000009-01 Oficina Admin.</t>
+        </is>
+      </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -2609,13 +2641,21 @@
           <t>Etapa N°1 al 4</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Fundo Zapallar — Etapa 1-4 y Etapa 5</t>
+        </is>
+      </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>1 placa</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr"/>
+          <t>2 placas</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>000027-03 Etapa N°5; 000027-04 Etapa N°1 al 4</t>
+        </is>
+      </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -2723,13 +2763,21 @@
           <t>Etapa N°5</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr"/>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Fundo Zapallar — Etapa 1-4 y Etapa 5</t>
+        </is>
+      </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>1 placa</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr"/>
+          <t>2 placas</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>000027-03 Etapa N°5; 000027-04 Etapa N°1 al 4</t>
+        </is>
+      </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -4727,7 +4775,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 11:28 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 11:33 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5068,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>28/08/2026 11:28 hora Chile</t>
+          <t>28/08/2026 11:33 hora Chile</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the equipment Excel with the confirmed Nido 3-plate cabinet.
Elementary, High School, and Teatro now share gabinete name, tipo, and node list; Drive Monitoreo/Control marks are kept.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -578,7 +578,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 28/08/2026 11:33 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
+          <t>Equipos vigentes al 28/08/2026 12:52 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
         </is>
       </c>
     </row>
@@ -3075,13 +3075,21 @@
           <t>Elementary</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr"/>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Nido de Águilas — Elementary / High School / Teatro</t>
+        </is>
+      </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr"/>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>000007-02 Teatro; 000007-03 Nido High School; 000007-04 Elementary</t>
+        </is>
+      </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3189,13 +3197,21 @@
           <t>Nido High School</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr"/>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Nido de Águilas — Elementary / High School / Teatro</t>
+        </is>
+      </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr"/>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>000007-02 Teatro; 000007-03 Nido High School; 000007-04 Elementary</t>
+        </is>
+      </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3303,13 +3319,21 @@
           <t>Teatro</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr"/>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Nido de Águilas — Elementary / High School / Teatro</t>
+        </is>
+      </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>000007-02 Teatro; 000007-03 Nido High School; 000007-04 Elementary</t>
+        </is>
+      </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -4775,7 +4799,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 11:33 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 12:52 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5092,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>28/08/2026 11:33 hora Chile</t>
+          <t>28/08/2026 12:52 hora Chile</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5152,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Complete con el desplegable: 1 a 5 placas. Ya vienen llenos los gabinetes confirmados (COPEC: 4 lavados; y matriz + riego + estanque).</t>
+          <t>Complete con el desplegable: 1 a 5 placas. Ya vienen llenos los gabinetes confirmados (COPEC, Fundo Zapallar etapas 1-4/5, Nido Elementary/High School/Teatro).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the Excel with Curauma rings, Andén 3-4, and Distrito de lujo cabinets.
Drive Monitoreo/Control marks are kept; the three Parque Arauco groups now have gabinete, tipo, and node lists filled.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
+++ b/reports/Puntos_En_Cero/Listado_Equipos_Vigentes_Puntos_En_Cero.xlsx
@@ -578,7 +578,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipos vigentes al 28/08/2026 12:52 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
+          <t>Equipos vigentes al 28/08/2026 13:04 (hora Chile). Complete Tipo gabinete (1 a 5 placas) y Nodos que contiene el gabinete. Los gabinetes ya confirmados (p. ej. COPEC lavados y matriz/riego/estanque) vienen llenos. Monitoreo y Control: Sí/No.</t>
         </is>
       </c>
     </row>
@@ -3517,13 +3517,21 @@
           <t>CUR Anillo Norte</t>
         </is>
       </c>
-      <c r="E77" s="6" t="inlineStr"/>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Curauma — Anillo Norte/Sur</t>
+        </is>
+      </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G77" s="6" t="inlineStr"/>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>000025-37 CUR Anillo Sur; 000025-38 CUR Anillo Norte</t>
+        </is>
+      </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3555,13 +3563,21 @@
           <t>CUR Anillo Sur</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr"/>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Curauma — Anillo Norte/Sur</t>
+        </is>
+      </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
           <t>2 placas</t>
         </is>
       </c>
-      <c r="G78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>000025-37 CUR Anillo Sur; 000025-38 CUR Anillo Norte</t>
+        </is>
+      </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3593,13 +3609,21 @@
           <t>Distrito de lujo DL</t>
         </is>
       </c>
-      <c r="E79" s="6" t="inlineStr"/>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Distrito de lujo</t>
+        </is>
+      </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>1 placa</t>
-        </is>
-      </c>
-      <c r="G79" s="6" t="inlineStr"/>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>000025-27 Distrito de lujo DL; 000025-35 PAK BAZAR GOURMET; 000025-36 PAK DL KENNEDY</t>
+        </is>
+      </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3669,13 +3693,21 @@
           <t>Impulsión Anden 3-4 Locales Gast.</t>
         </is>
       </c>
-      <c r="E81" s="6" t="inlineStr"/>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Andén 3-4</t>
+        </is>
+      </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>000025-20 Impulsión Anden 3-4 Matriz Principal; 000025-21 Impulsión Anden 3-4 Locales Gast.; 000025-29 Impulsión Anden 3-4 Restaurante</t>
+        </is>
+      </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3707,13 +3739,21 @@
           <t>Impulsión Anden 3-4 Matriz Principal</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr"/>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Andén 3-4</t>
+        </is>
+      </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>000025-20 Impulsión Anden 3-4 Matriz Principal; 000025-21 Impulsión Anden 3-4 Locales Gast.; 000025-29 Impulsión Anden 3-4 Restaurante</t>
+        </is>
+      </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3745,13 +3785,21 @@
           <t>Impulsión Anden 3-4 Restaurante</t>
         </is>
       </c>
-      <c r="E83" s="6" t="inlineStr"/>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Andén 3-4</t>
+        </is>
+      </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
           <t>3 placas</t>
         </is>
       </c>
-      <c r="G83" s="6" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>000025-20 Impulsión Anden 3-4 Matriz Principal; 000025-21 Impulsión Anden 3-4 Locales Gast.; 000025-29 Impulsión Anden 3-4 Restaurante</t>
+        </is>
+      </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -4049,13 +4097,21 @@
           <t>PAK BAZAR GOURMET</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr"/>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Distrito de lujo</t>
+        </is>
+      </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>1 placa</t>
-        </is>
-      </c>
-      <c r="G91" s="6" t="inlineStr"/>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>000025-27 Distrito de lujo DL; 000025-35 PAK BAZAR GOURMET; 000025-36 PAK DL KENNEDY</t>
+        </is>
+      </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -4087,13 +4143,21 @@
           <t>PAK DL KENNEDY</t>
         </is>
       </c>
-      <c r="E92" s="6" t="inlineStr"/>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>Parque Arauco Kennedy — Distrito de lujo</t>
+        </is>
+      </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
-          <t>1 placa</t>
-        </is>
-      </c>
-      <c r="G92" s="6" t="inlineStr"/>
+          <t>3 placas</t>
+        </is>
+      </c>
+      <c r="G92" s="6" t="inlineStr">
+        <is>
+          <t>000025-27 Distrito de lujo DL; 000025-35 PAK BAZAR GOURMET; 000025-36 PAK DL KENNEDY</t>
+        </is>
+      </c>
       <c r="H92" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -4799,7 +4863,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 12:52 hora Chile.</t>
+          <t>Cantidad de equipos vigentes incluidos en el reporte matinal de puntos en cero. Generado 28/08/2026 13:04 hora Chile.</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5156,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>28/08/2026 12:52 hora Chile</t>
+          <t>28/08/2026 13:04 hora Chile</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5216,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Complete con el desplegable: 1 a 5 placas. Ya vienen llenos los gabinetes confirmados (COPEC, Fundo Zapallar etapas 1-4/5, Nido Elementary/High School/Teatro).</t>
+          <t>Complete con el desplegable: 1 a 5 placas. Ya vienen llenos los gabinetes confirmados (COPEC, Fundo Zapallar etapas 1-4/5, Nido Elementary/High School/Teatro, PA Curauma anillos, PA Kennedy Andén 3-4 y Distrito de lujo).</t>
         </is>
       </c>
     </row>

</xml_diff>